<commit_message>
Update trabalho de matematica dados.xlsx
</commit_message>
<xml_diff>
--- a/trabalho de matematica dados.xlsx
+++ b/trabalho de matematica dados.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pedro Vitor Ortiz\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pedro Vitor Ortiz\Downloads\Documents\GitHub\trabalho.Funcoes.trigonometricas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79267D49-6642-41AD-977F-CCE7346FF3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91937B7-74F4-4796-BF64-3CF69F299330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{689BB34E-0E18-4B3F-9640-5C22EDA1B746}"/>
   </bookViews>
@@ -629,6 +629,7 @@
         <v>277</v>
       </c>
       <c r="C2" s="6">
+        <f>1/B2</f>
         <v>3.6101083032490976E-3</v>
       </c>
       <c r="D2" s="13" t="s">
@@ -642,7 +643,8 @@
       <c r="B3" s="8">
         <v>293</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="6">
+        <f t="shared" ref="C3:C12" si="0">1/B3</f>
         <v>3.4129692832764505E-3</v>
       </c>
       <c r="D3"/>
@@ -655,6 +657,7 @@
         <v>311</v>
       </c>
       <c r="C4" s="6">
+        <f t="shared" si="0"/>
         <v>3.2154340836012861E-3</v>
       </c>
       <c r="D4" s="13" t="s">
@@ -668,7 +671,8 @@
       <c r="B5" s="8">
         <v>329</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="6">
+        <f t="shared" si="0"/>
         <v>3.0395136778115501E-3</v>
       </c>
       <c r="D5" s="14" t="s">
@@ -683,6 +687,7 @@
         <v>349</v>
       </c>
       <c r="C6" s="6">
+        <f t="shared" si="0"/>
         <v>2.8653295128939827E-3</v>
       </c>
       <c r="D6"/>
@@ -694,7 +699,8 @@
       <c r="B7" s="8">
         <v>369</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="6">
+        <f t="shared" si="0"/>
         <v>2.7100271002710027E-3</v>
       </c>
       <c r="D7" s="2"/>
@@ -707,6 +713,7 @@
         <v>391</v>
       </c>
       <c r="C8" s="6">
+        <f t="shared" si="0"/>
         <v>2.5575447570332483E-3</v>
       </c>
       <c r="D8" s="2"/>
@@ -719,6 +726,7 @@
         <v>415</v>
       </c>
       <c r="C9" s="6">
+        <f t="shared" si="0"/>
         <v>2.4096385542168677E-3</v>
       </c>
       <c r="D9"/>
@@ -731,6 +739,7 @@
         <v>440</v>
       </c>
       <c r="C10" s="6">
+        <f t="shared" si="0"/>
         <v>2.2727272727272726E-3</v>
       </c>
       <c r="D10" s="2"/>
@@ -743,6 +752,7 @@
         <v>466</v>
       </c>
       <c r="C11" s="6">
+        <f t="shared" si="0"/>
         <v>2.1459227467811159E-3</v>
       </c>
       <c r="D11"/>
@@ -755,6 +765,7 @@
         <v>493</v>
       </c>
       <c r="C12" s="6">
+        <f t="shared" si="0"/>
         <v>2.0283975659229209E-3</v>
       </c>
       <c r="D12"/>

</xml_diff>

<commit_message>
colocando o novo codigo
</commit_message>
<xml_diff>
--- a/trabalho de matematica dados.xlsx
+++ b/trabalho de matematica dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pedro Vitor Ortiz\Downloads\Documents\GitHub\trabalho.Funcoes.trigonometricas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC911839-DD05-44DE-90FA-B05222A34007}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60ACB2C8-120C-42AF-80A7-394707039F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{689BB34E-0E18-4B3F-9640-5C22EDA1B746}"/>
   </bookViews>
@@ -37,17 +37,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>notas</t>
   </si>
   <si>
-    <t>hetz</t>
-  </si>
-  <si>
-    <t>periodo em segundos</t>
-  </si>
-  <si>
     <t>C# 3</t>
   </si>
   <si>
@@ -96,7 +90,22 @@
     <t>data de acesso final:13/09/2026</t>
   </si>
   <si>
-    <t>periodo em milesegundois</t>
+    <t>Hertz</t>
+  </si>
+  <si>
+    <t>período em segundos</t>
+  </si>
+  <si>
+    <t>período em milissegundos</t>
+  </si>
+  <si>
+    <t>máximo</t>
+  </si>
+  <si>
+    <t>mínimo</t>
+  </si>
+  <si>
+    <t>λ</t>
   </si>
 </sst>
 </file>
@@ -611,37 +620,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8992B49F-851A-4F89-B8AB-AAFD4B766DDD}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="58.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="5" max="5" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" style="1"/>
+    <col min="8" max="8" width="59.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="D1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" s="7">
         <v>277</v>
@@ -654,30 +675,50 @@
         <f>C2*1000</f>
         <v>3.6101083032490977</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E2" s="7">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7">
+        <v>-1</v>
+      </c>
+      <c r="G2" s="7">
+        <f>344/B2</f>
+        <v>1.2418772563176896</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" s="9">
         <v>293</v>
       </c>
       <c r="C3" s="9">
-        <f t="shared" ref="C3:D12" si="0">1/B3</f>
+        <f t="shared" ref="C3:C12" si="0">1/B3</f>
         <v>3.4129692832764505E-3</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="9">
         <f t="shared" ref="D3:D12" si="1">C3*1000</f>
         <v>3.4129692832764507</v>
       </c>
-      <c r="E3"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E3" s="9">
+        <v>1</v>
+      </c>
+      <c r="F3" s="9">
+        <v>-1</v>
+      </c>
+      <c r="G3" s="7">
+        <f t="shared" ref="G3:G12" si="2">344/B3</f>
+        <v>1.1740614334470989</v>
+      </c>
+      <c r="H3"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4" s="7">
         <v>311</v>
@@ -690,13 +731,23 @@
         <f t="shared" si="1"/>
         <v>3.215434083601286</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E4" s="7">
+        <v>1</v>
+      </c>
+      <c r="F4" s="7">
+        <v>-1</v>
+      </c>
+      <c r="G4" s="7">
+        <f t="shared" si="2"/>
+        <v>1.1061093247588425</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5" s="9">
         <v>329</v>
@@ -705,17 +756,27 @@
         <f t="shared" si="0"/>
         <v>3.0395136778115501E-3</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="9">
         <f t="shared" si="1"/>
         <v>3.0395136778115504</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E5" s="9">
+        <v>1</v>
+      </c>
+      <c r="F5" s="9">
+        <v>-1</v>
+      </c>
+      <c r="G5" s="7">
+        <f t="shared" si="2"/>
+        <v>1.0455927051671732</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" s="7">
         <v>349</v>
@@ -728,13 +789,23 @@
         <f t="shared" si="1"/>
         <v>2.8653295128939829</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E6" s="7">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7">
+        <v>-1</v>
+      </c>
+      <c r="G6" s="7">
+        <f t="shared" si="2"/>
+        <v>0.98567335243553011</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7" s="9">
         <v>369</v>
@@ -743,15 +814,25 @@
         <f t="shared" si="0"/>
         <v>2.7100271002710027E-3</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="10">
         <f t="shared" si="1"/>
         <v>2.7100271002710028</v>
       </c>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E7" s="10">
+        <v>1</v>
+      </c>
+      <c r="F7" s="10">
+        <v>-1</v>
+      </c>
+      <c r="G7" s="7">
+        <f t="shared" si="2"/>
+        <v>0.9322493224932249</v>
+      </c>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B8" s="11">
         <v>391</v>
@@ -764,11 +845,21 @@
         <f t="shared" si="1"/>
         <v>2.5575447570332481</v>
       </c>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E8" s="7">
+        <v>1</v>
+      </c>
+      <c r="F8" s="7">
+        <v>-1</v>
+      </c>
+      <c r="G8" s="7">
+        <f t="shared" si="2"/>
+        <v>0.87979539641943738</v>
+      </c>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="12">
         <v>415</v>
@@ -777,15 +868,25 @@
         <f t="shared" si="0"/>
         <v>2.4096385542168677E-3</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="10">
         <f t="shared" si="1"/>
         <v>2.4096385542168677</v>
       </c>
-      <c r="E9"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E9" s="10">
+        <v>1</v>
+      </c>
+      <c r="F9" s="10">
+        <v>-1</v>
+      </c>
+      <c r="G9" s="7">
+        <f t="shared" si="2"/>
+        <v>0.82891566265060246</v>
+      </c>
+      <c r="H9"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10" s="11">
         <v>440</v>
@@ -798,11 +899,21 @@
         <f t="shared" si="1"/>
         <v>2.2727272727272725</v>
       </c>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E10" s="7">
+        <v>1</v>
+      </c>
+      <c r="F10" s="7">
+        <v>-1</v>
+      </c>
+      <c r="G10" s="7">
+        <f t="shared" si="2"/>
+        <v>0.78181818181818186</v>
+      </c>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11" s="12">
         <v>466</v>
@@ -811,15 +922,25 @@
         <f t="shared" si="0"/>
         <v>2.1459227467811159E-3</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="10">
         <f t="shared" si="1"/>
         <v>2.1459227467811157</v>
       </c>
-      <c r="E11"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E11" s="10">
+        <v>1</v>
+      </c>
+      <c r="F11" s="10">
+        <v>-1</v>
+      </c>
+      <c r="G11" s="7">
+        <f t="shared" si="2"/>
+        <v>0.7381974248927039</v>
+      </c>
+      <c r="H11"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B12" s="11">
         <v>493</v>
@@ -832,27 +953,37 @@
         <f t="shared" si="1"/>
         <v>2.028397565922921</v>
       </c>
-      <c r="E12"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E12" s="7">
+        <v>1</v>
+      </c>
+      <c r="F12" s="7">
+        <v>-1</v>
+      </c>
+      <c r="G12" s="7">
+        <f t="shared" si="2"/>
+        <v>0.69776876267748478</v>
+      </c>
+      <c r="H12"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13"/>
       <c r="B13"/>
       <c r="C13"/>
-      <c r="E13"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H13"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14"/>
       <c r="B14"/>
       <c r="C14"/>
-      <c r="E14"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="H14"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15"/>
       <c r="B15"/>
       <c r="C15"/>
       <c r="E15"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16"/>
       <c r="B16"/>
       <c r="C16"/>
@@ -879,7 +1010,7 @@
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="E5" r:id="rId1" xr:uid="{CACA5D8B-9DF6-4E5B-BC8D-1C82F77403EE}"/>
+    <hyperlink ref="H5" r:id="rId1" xr:uid="{CACA5D8B-9DF6-4E5B-BC8D-1C82F77403EE}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>

</xml_diff>